<commit_message>
update code feedback29-4-26.ipynb so that the same unit from third analysis can be combined together
</commit_message>
<xml_diff>
--- a/Hasil Analisa Feedback 29-4-26.xlsx
+++ b/Hasil Analisa Feedback 29-4-26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Downloads\SPIL\bbm\Analisa BBM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1215A02-1018-42B1-98AD-C8A7B72C06F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17AE74F3-E78C-4B57-BF8A-8952657B72EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A1_Ringkasan_MAPE_Over35" sheetId="1" r:id="rId1"/>
@@ -26,16 +26,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">A1_Ringkasan_MAPE_Over35!$A$1:$H$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">A2_Unit_Dikecualikan!$A$1:$C$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">A3_Detail_Bulanan_Anomali!$A$1:$F$577</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">A3_Semua_Anomali!$A$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">A3_Semua_Anomali!$A$1:$J$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">A3_TipeA_Streak_3Bulan!$A$1:$J$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">A3_TipeB_Terisolir!$A$1:$J$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">A3_TipeB_Terisolir!$A$1:$J$14</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5820" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5795" uniqueCount="257">
   <si>
     <t>EQUIP NAME</t>
   </si>
@@ -658,9 +658,6 @@
     <t>2023-05</t>
   </si>
   <si>
-    <t>2023-06</t>
-  </si>
-  <si>
     <t>2023-09</t>
   </si>
   <si>
@@ -691,46 +688,43 @@
     <t>2024-06</t>
   </si>
   <si>
+    <t>2023-06</t>
+  </si>
+  <si>
     <t>2024-04</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2022-03, 2022-04) HM=0. 2 bulan sesudah (2022-06, 2022-07) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2022-05) di tengah periode tidak aktif. 2 bulan sebelum: (2022-03, 2022-04). 2 bulan sesudah: (2022-06, 2022-07).</t>
   </si>
   <si>
     <t>HM=0 &amp; LITER&gt;0 selama 3 bulan berturut-turut</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2025-04, 2025-05) HM=0. 2 bulan sesudah (2025-07, 2025-08) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 2 bulan terisolir (2025-06, 2025-07) di tengah periode tidak aktif. 2 bulan sebelum: (2025-04, 2025-05). 2 bulan sesudah: (2025-08, 2025-09).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2025-05, 2025-06) HM=0. 2 bulan sesudah (2025-08, 2025-09) HM=0.</t>
-  </si>
-  <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2022-01, 2022-02) HM=0. 2 bulan sesudah (2022-04, 2022-05) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2022-03) di tengah periode tidak aktif. 2 bulan sebelum: (2022-01, 2022-02). 2 bulan sesudah: (2022-04, 2022-05).</t>
   </si>
   <si>
     <t>HM=0 &amp; LITER&gt;0 selama 18 bulan berturut-turut</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2022-07, 2022-08) HM=0. 2 bulan sesudah (2022-10, 2022-11) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2022-09) di tengah periode tidak aktif. 2 bulan sebelum: (2022-07, 2022-08). 2 bulan sesudah: (2022-10, 2022-11).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2023-03, 2023-04) HM=0. 2 bulan sesudah (2023-06, 2023-07) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 2 bulan terisolir (2023-05, 2023-06) di tengah periode tidak aktif. 2 bulan sebelum: (2023-03, 2023-04). 2 bulan sesudah: (2023-07, 2023-08).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2023-04, 2023-05) HM=0. 2 bulan sesudah (2023-07, 2023-08) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2024-01) di tengah periode tidak aktif. 2 bulan sebelum: (2023-11, 2023-12). 2 bulan sesudah: (2024-02, 2024-03).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2023-11, 2023-12) HM=0. 2 bulan sesudah (2024-02, 2024-03) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2024-07) di tengah periode tidak aktif. 2 bulan sebelum: (2024-05, 2024-06). 2 bulan sesudah: (2024-08, 2024-09).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2024-05, 2024-06) HM=0. 2 bulan sesudah (2024-08, 2024-09) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2024-10) di tengah periode tidak aktif. 2 bulan sebelum: (2024-08, 2024-09). 2 bulan sesudah: (2024-11, 2024-12).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2024-08, 2024-09) HM=0. 2 bulan sesudah (2024-11, 2024-12) HM=0.</t>
-  </si>
-  <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2025-01, 2025-02) HM=0. 2 bulan sesudah (2025-04, 2025-05) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2025-03) di tengah periode tidak aktif. 2 bulan sebelum: (2025-01, 2025-02). 2 bulan sesudah: (2025-04, 2025-05).</t>
   </si>
   <si>
     <t>HM=0 &amp; LITER&gt;0 selama 14 bulan berturut-turut</t>
@@ -739,13 +733,16 @@
     <t>HM=0 &amp; LITER&gt;0 selama 13 bulan berturut-turut</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2024-09, 2024-10) HM=0. 2 bulan sesudah (2024-12, 2025-01) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2024-11) di tengah periode tidak aktif. 2 bulan sebelum: (2024-09, 2024-10). 2 bulan sesudah: (2024-12, 2025-01).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2023-09, 2023-10) HM=0. 2 bulan sesudah (2023-12, 2024-01) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2025-07) di tengah periode tidak aktif. 2 bulan sebelum: (2025-05, 2025-06). 2 bulan sesudah: (2025-08, 2025-09).</t>
   </si>
   <si>
-    <t>HM=0 &amp; LITER&gt;0 di bulan ini. 2 bulan sebelum (2024-01, 2024-02) HM=0. 2 bulan sesudah (2024-04, 2024-05) HM=0.</t>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2023-11) di tengah periode tidak aktif. 2 bulan sebelum: (2023-09, 2023-10). 2 bulan sesudah: (2023-12, 2024-01).</t>
+  </si>
+  <si>
+    <t>HM=0 &amp; LITER&gt;0 selama 1 bulan terisolir (2024-03) di tengah periode tidak aktif. 2 bulan sebelum: (2024-01, 2024-02). 2 bulan sesudah: (2024-04, 2024-05).</t>
   </si>
   <si>
     <t>NAMA_MASTER</t>
@@ -809,9 +806,6 @@
   </si>
   <si>
     <t>2024-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -3064,11 +3058,11 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="0" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.5703125" bestFit="1" customWidth="1"/>
@@ -35046,8 +35040,7 @@
   <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="31.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="51.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -35796,7 +35789,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -35808,7 +35801,7 @@
     <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="103" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="147.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -35845,63 +35838,63 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>107</v>
+        <v>194</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>194</v>
       </c>
       <c r="C2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>100</v>
+        <v>470</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="I2">
-        <v>100</v>
+        <v>156.66999999999999</v>
       </c>
       <c r="J2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>112</v>
       </c>
       <c r="B3" t="s">
-        <v>194</v>
+        <v>112</v>
       </c>
       <c r="C3" t="s">
         <v>198</v>
       </c>
       <c r="D3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E3" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="F3">
         <v>3</v>
       </c>
       <c r="G3">
-        <v>470</v>
+        <v>90</v>
       </c>
       <c r="H3">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>156.66999999999999</v>
+        <v>30</v>
       </c>
       <c r="J3" t="s">
         <v>220</v>
@@ -35909,31 +35902,31 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>195</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
+        <v>196</v>
       </c>
       <c r="C4" t="s">
         <v>198</v>
       </c>
       <c r="D4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E4" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="F4">
         <v>3</v>
       </c>
       <c r="G4">
-        <v>90</v>
+        <v>5712.05</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="I4">
-        <v>30</v>
+        <v>1904.02</v>
       </c>
       <c r="J4" t="s">
         <v>220</v>
@@ -35941,226 +35934,226 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>195</v>
+        <v>119</v>
       </c>
       <c r="B5" t="s">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
         <v>198</v>
       </c>
       <c r="D5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G5">
-        <v>5712.05</v>
+        <v>5825</v>
       </c>
       <c r="H5">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="I5">
-        <v>1904.02</v>
+        <v>323.61</v>
       </c>
       <c r="J5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>207</v>
       </c>
       <c r="E6" t="s">
-        <v>99</v>
+        <v>213</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6">
-        <v>25</v>
+        <v>395</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I6">
-        <v>25</v>
+        <v>131.66999999999999</v>
       </c>
       <c r="J6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E7" t="s">
-        <v>100</v>
+        <v>202</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G7">
-        <v>25</v>
+        <v>24083</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>251</v>
       </c>
       <c r="I7">
-        <v>25</v>
+        <v>1720.21</v>
       </c>
       <c r="J7" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D8" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="E8" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G8">
-        <v>10</v>
+        <v>18765</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>162</v>
       </c>
       <c r="I8">
-        <v>10</v>
+        <v>1443.46</v>
       </c>
       <c r="J8" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E9" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="F9">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>5825</v>
+        <v>100</v>
       </c>
       <c r="H9">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>323.61</v>
+        <v>100</v>
       </c>
       <c r="J9" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
         <v>197</v>
       </c>
       <c r="D10" t="s">
-        <v>205</v>
+        <v>99</v>
       </c>
       <c r="E10" t="s">
-        <v>205</v>
+        <v>100</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="J10" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C11" t="s">
         <v>197</v>
       </c>
       <c r="D11" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E11" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
       <c r="I11">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="J11" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -36174,25 +36167,25 @@
         <v>197</v>
       </c>
       <c r="D12" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E12" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="J12" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -36203,28 +36196,28 @@
         <v>120</v>
       </c>
       <c r="C13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E13" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>395</v>
+        <v>170</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I13">
-        <v>131.66999999999999</v>
+        <v>85</v>
       </c>
       <c r="J13" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -36238,10 +36231,10 @@
         <v>197</v>
       </c>
       <c r="D14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -36256,7 +36249,7 @@
         <v>80</v>
       </c>
       <c r="J14" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -36270,10 +36263,10 @@
         <v>197</v>
       </c>
       <c r="D15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -36288,7 +36281,7 @@
         <v>200</v>
       </c>
       <c r="J15" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -36302,10 +36295,10 @@
         <v>197</v>
       </c>
       <c r="D16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -36320,7 +36313,7 @@
         <v>160</v>
       </c>
       <c r="J16" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -36352,36 +36345,36 @@
         <v>89.98</v>
       </c>
       <c r="J17" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>172</v>
       </c>
       <c r="B18" t="s">
-        <v>121</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D18" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="E18" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="F18">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G18">
-        <v>24083</v>
+        <v>12</v>
       </c>
       <c r="H18">
-        <v>251</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>1720.21</v>
+        <v>12</v>
       </c>
       <c r="J18" t="s">
         <v>232</v>
@@ -36389,31 +36382,31 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>121</v>
+        <v>172</v>
       </c>
       <c r="B19" t="s">
-        <v>121</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D19" t="s">
-        <v>212</v>
+        <v>100</v>
       </c>
       <c r="E19" t="s">
-        <v>218</v>
+        <v>100</v>
       </c>
       <c r="F19">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G19">
-        <v>18765</v>
+        <v>27.79</v>
       </c>
       <c r="H19">
-        <v>162</v>
+        <v>1</v>
       </c>
       <c r="I19">
-        <v>1443.46</v>
+        <v>27.79</v>
       </c>
       <c r="J19" t="s">
         <v>233</v>
@@ -36421,10 +36414,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>172</v>
+        <v>49</v>
       </c>
       <c r="B20" t="s">
-        <v>172</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
         <v>197</v>
@@ -36439,13 +36432,13 @@
         <v>1</v>
       </c>
       <c r="G20">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H20">
         <v>1</v>
       </c>
       <c r="I20">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="J20" t="s">
         <v>234</v>
@@ -36453,104 +36446,40 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="B21" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="C21" t="s">
         <v>197</v>
       </c>
       <c r="D21" t="s">
-        <v>100</v>
+        <v>214</v>
       </c>
       <c r="E21" t="s">
-        <v>100</v>
+        <v>214</v>
       </c>
       <c r="F21">
         <v>1</v>
       </c>
       <c r="G21">
-        <v>27.79</v>
+        <v>200</v>
       </c>
       <c r="H21">
         <v>1</v>
       </c>
       <c r="I21">
-        <v>27.79</v>
+        <v>200</v>
       </c>
       <c r="J21" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" t="s">
-        <v>197</v>
-      </c>
-      <c r="D22" t="s">
-        <v>214</v>
-      </c>
-      <c r="E22" t="s">
-        <v>214</v>
-      </c>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22">
-        <v>50</v>
-      </c>
-      <c r="H22">
-        <v>1</v>
-      </c>
-      <c r="I22">
-        <v>50</v>
-      </c>
-      <c r="J22" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>122</v>
-      </c>
-      <c r="B23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C23" t="s">
-        <v>197</v>
-      </c>
-      <c r="D23" t="s">
-        <v>215</v>
-      </c>
-      <c r="E23" t="s">
-        <v>215</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>200</v>
-      </c>
-      <c r="H23">
-        <v>1</v>
-      </c>
-      <c r="I23">
-        <v>200</v>
-      </c>
-      <c r="J23" t="s">
-        <v>236</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J23" xr:uid="{00000000-0001-0000-0300-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J23">
-      <sortCondition ref="A1:A23"/>
+  <autoFilter ref="A1:J21" xr:uid="{00000000-0001-0000-0300-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J21">
+      <sortCondition ref="C1:C21"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -36563,8 +36492,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="0" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.140625" bestFit="1" customWidth="1"/>
@@ -36652,7 +36581,7 @@
         <v>201</v>
       </c>
       <c r="E3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F3">
         <v>3</v>
@@ -36684,7 +36613,7 @@
         <v>202</v>
       </c>
       <c r="E4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -36716,7 +36645,7 @@
         <v>204</v>
       </c>
       <c r="E5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F5">
         <v>18</v>
@@ -36731,7 +36660,7 @@
         <v>323.61</v>
       </c>
       <c r="J5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -36745,10 +36674,10 @@
         <v>198</v>
       </c>
       <c r="D6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F6">
         <v>3</v>
@@ -36795,7 +36724,7 @@
         <v>1720.21</v>
       </c>
       <c r="J7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -36809,7 +36738,7 @@
         <v>198</v>
       </c>
       <c r="D8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E8" t="s">
         <v>218</v>
@@ -36827,7 +36756,7 @@
         <v>1443.46</v>
       </c>
       <c r="J8" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -36842,19 +36771,19 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="103" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="147.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -36935,16 +36864,16 @@
         <v>99</v>
       </c>
       <c r="E3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3">
         <v>25</v>
@@ -36955,31 +36884,31 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="C4" t="s">
         <v>197</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>203</v>
       </c>
       <c r="E4" t="s">
-        <v>100</v>
+        <v>203</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="I4">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="J4" t="s">
         <v>222</v>
@@ -36987,34 +36916,34 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
         <v>197</v>
       </c>
       <c r="D5" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E5" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="H5">
         <v>1</v>
       </c>
       <c r="I5">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="J5" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -37028,22 +36957,22 @@
         <v>197</v>
       </c>
       <c r="D6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E6" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>150</v>
+        <v>85</v>
       </c>
       <c r="J6" t="s">
         <v>225</v>
@@ -37060,25 +36989,25 @@
         <v>197</v>
       </c>
       <c r="D7" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="E7" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="J7" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -37092,25 +37021,25 @@
         <v>197</v>
       </c>
       <c r="D8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F8">
         <v>1</v>
       </c>
       <c r="G8">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="J8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -37124,25 +37053,25 @@
         <v>197</v>
       </c>
       <c r="D9" t="s">
-        <v>209</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>209</v>
+        <v>96</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9">
-        <v>80</v>
+        <v>89.98</v>
       </c>
       <c r="H9">
         <v>1</v>
       </c>
       <c r="I9">
-        <v>80</v>
+        <v>89.98</v>
       </c>
       <c r="J9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -37156,97 +37085,97 @@
         <v>197</v>
       </c>
       <c r="D10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="H10">
         <v>1</v>
       </c>
       <c r="I10">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="J10" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="B11" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
         <v>197</v>
       </c>
       <c r="D11" t="s">
-        <v>211</v>
+        <v>100</v>
       </c>
       <c r="E11" t="s">
-        <v>211</v>
+        <v>100</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11">
-        <v>160</v>
+        <v>27.79</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
       <c r="I11">
-        <v>160</v>
+        <v>27.79</v>
       </c>
       <c r="J11" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="B12" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
         <v>197</v>
       </c>
       <c r="D12" t="s">
-        <v>96</v>
+        <v>212</v>
       </c>
       <c r="E12" t="s">
-        <v>96</v>
+        <v>212</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12">
-        <v>89.98</v>
+        <v>12</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12">
-        <v>89.98</v>
+        <v>12</v>
       </c>
       <c r="J12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>172</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
         <v>197</v>
@@ -37261,13 +37190,13 @@
         <v>1</v>
       </c>
       <c r="G13">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
       <c r="I13">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="J13" t="s">
         <v>234</v>
@@ -37275,104 +37204,40 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="C14" t="s">
         <v>197</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>214</v>
       </c>
       <c r="E14" t="s">
-        <v>100</v>
+        <v>214</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14">
-        <v>27.79</v>
+        <v>200</v>
       </c>
       <c r="H14">
         <v>1</v>
       </c>
       <c r="I14">
-        <v>27.79</v>
+        <v>200</v>
       </c>
       <c r="J14" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>49</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" t="s">
-        <v>197</v>
-      </c>
-      <c r="D15" t="s">
-        <v>214</v>
-      </c>
-      <c r="E15" t="s">
-        <v>214</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15">
-        <v>50</v>
-      </c>
-      <c r="H15">
-        <v>1</v>
-      </c>
-      <c r="I15">
-        <v>50</v>
-      </c>
-      <c r="J15" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>122</v>
-      </c>
-      <c r="B16" t="s">
-        <v>122</v>
-      </c>
-      <c r="C16" t="s">
-        <v>197</v>
-      </c>
-      <c r="D16" t="s">
-        <v>215</v>
-      </c>
-      <c r="E16" t="s">
-        <v>215</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
-      <c r="G16">
-        <v>200</v>
-      </c>
-      <c r="H16">
-        <v>1</v>
-      </c>
-      <c r="I16">
-        <v>200</v>
-      </c>
-      <c r="J16" t="s">
-        <v>236</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J16" xr:uid="{00000000-0001-0000-0500-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J16">
-      <sortCondition ref="A1:A16"/>
+  <autoFilter ref="A1:J14" xr:uid="{00000000-0001-0000-0500-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J14">
+      <sortCondition ref="A1:A14"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37381,7 +37246,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:I577"/>
+  <dimension ref="A1:F577"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -37397,19 +37262,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -37440,7 +37305,7 @@
         <v>107</v>
       </c>
       <c r="C3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -37480,7 +37345,7 @@
         <v>107</v>
       </c>
       <c r="C5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -37520,7 +37385,7 @@
         <v>107</v>
       </c>
       <c r="C7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -37540,7 +37405,7 @@
         <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -37560,7 +37425,7 @@
         <v>107</v>
       </c>
       <c r="C9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -37620,7 +37485,7 @@
         <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -37640,7 +37505,7 @@
         <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -37700,7 +37565,7 @@
         <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -37712,7 +37577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>107</v>
       </c>
@@ -37720,7 +37585,7 @@
         <v>107</v>
       </c>
       <c r="C17" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -37731,11 +37596,8 @@
       <c r="F17">
         <v>0</v>
       </c>
-      <c r="I17" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>107</v>
       </c>
@@ -37755,7 +37617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>107</v>
       </c>
@@ -37763,7 +37625,7 @@
         <v>107</v>
       </c>
       <c r="C19" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -37775,7 +37637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>107</v>
       </c>
@@ -37783,7 +37645,7 @@
         <v>107</v>
       </c>
       <c r="C20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -37795,7 +37657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>107</v>
       </c>
@@ -37803,7 +37665,7 @@
         <v>107</v>
       </c>
       <c r="C21" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -37815,7 +37677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>107</v>
       </c>
@@ -37823,7 +37685,7 @@
         <v>107</v>
       </c>
       <c r="C22" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -37835,7 +37697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>107</v>
       </c>
@@ -37843,7 +37705,7 @@
         <v>107</v>
       </c>
       <c r="C23" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -37855,7 +37717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>107</v>
       </c>
@@ -37863,7 +37725,7 @@
         <v>107</v>
       </c>
       <c r="C24" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -37875,7 +37737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>107</v>
       </c>
@@ -37883,7 +37745,7 @@
         <v>107</v>
       </c>
       <c r="C25" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -37895,7 +37757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>107</v>
       </c>
@@ -37903,7 +37765,7 @@
         <v>107</v>
       </c>
       <c r="C26" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -37915,7 +37777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>107</v>
       </c>
@@ -37923,7 +37785,7 @@
         <v>107</v>
       </c>
       <c r="C27" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -37935,7 +37797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>107</v>
       </c>
@@ -37943,7 +37805,7 @@
         <v>107</v>
       </c>
       <c r="C28" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -37955,7 +37817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>107</v>
       </c>
@@ -37975,7 +37837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>107</v>
       </c>
@@ -37983,7 +37845,7 @@
         <v>107</v>
       </c>
       <c r="C30" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -37995,7 +37857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>107</v>
       </c>
@@ -38003,7 +37865,7 @@
         <v>107</v>
       </c>
       <c r="C31" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -38015,7 +37877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>107</v>
       </c>
@@ -38023,7 +37885,7 @@
         <v>107</v>
       </c>
       <c r="C32" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D32">
         <v>127</v>
@@ -38043,7 +37905,7 @@
         <v>107</v>
       </c>
       <c r="C33" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D33">
         <v>96</v>
@@ -38063,7 +37925,7 @@
         <v>107</v>
       </c>
       <c r="C34" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D34">
         <v>145</v>
@@ -38083,7 +37945,7 @@
         <v>107</v>
       </c>
       <c r="C35" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D35">
         <v>153</v>
@@ -38103,7 +37965,7 @@
         <v>107</v>
       </c>
       <c r="C36" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D36">
         <v>60</v>
@@ -38123,7 +37985,7 @@
         <v>107</v>
       </c>
       <c r="C37" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D37">
         <v>34</v>
@@ -38403,7 +38265,7 @@
         <v>194</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D51" s="3">
         <v>0</v>
@@ -38443,7 +38305,7 @@
         <v>194</v>
       </c>
       <c r="C53" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D53">
         <v>27</v>
@@ -38483,7 +38345,7 @@
         <v>194</v>
       </c>
       <c r="C55" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D55">
         <v>41</v>
@@ -38503,7 +38365,7 @@
         <v>194</v>
       </c>
       <c r="C56" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D56">
         <v>29</v>
@@ -38523,7 +38385,7 @@
         <v>194</v>
       </c>
       <c r="C57" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D57">
         <v>190</v>
@@ -38583,7 +38445,7 @@
         <v>194</v>
       </c>
       <c r="C60" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D60">
         <v>130</v>
@@ -38603,7 +38465,7 @@
         <v>194</v>
       </c>
       <c r="C61" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D61">
         <v>101</v>
@@ -38663,7 +38525,7 @@
         <v>194</v>
       </c>
       <c r="C64" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D64">
         <v>110</v>
@@ -38683,7 +38545,7 @@
         <v>194</v>
       </c>
       <c r="C65" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D65">
         <v>69</v>
@@ -38723,7 +38585,7 @@
         <v>194</v>
       </c>
       <c r="C67" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D67">
         <v>143</v>
@@ -38743,7 +38605,7 @@
         <v>194</v>
       </c>
       <c r="C68" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D68">
         <v>140</v>
@@ -38763,7 +38625,7 @@
         <v>194</v>
       </c>
       <c r="C69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D69">
         <v>138</v>
@@ -38783,7 +38645,7 @@
         <v>194</v>
       </c>
       <c r="C70" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D70">
         <v>149</v>
@@ -38803,7 +38665,7 @@
         <v>194</v>
       </c>
       <c r="C71" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D71">
         <v>165</v>
@@ -38823,7 +38685,7 @@
         <v>194</v>
       </c>
       <c r="C72" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D72">
         <v>154</v>
@@ -38843,7 +38705,7 @@
         <v>194</v>
       </c>
       <c r="C73" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D73">
         <v>135</v>
@@ -38863,7 +38725,7 @@
         <v>194</v>
       </c>
       <c r="C74" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D74">
         <v>120</v>
@@ -38883,7 +38745,7 @@
         <v>194</v>
       </c>
       <c r="C75" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D75">
         <v>133</v>
@@ -38903,7 +38765,7 @@
         <v>194</v>
       </c>
       <c r="C76" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D76">
         <v>114</v>
@@ -38943,7 +38805,7 @@
         <v>194</v>
       </c>
       <c r="C78" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D78">
         <v>109</v>
@@ -38963,7 +38825,7 @@
         <v>194</v>
       </c>
       <c r="C79" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D79">
         <v>86</v>
@@ -38983,7 +38845,7 @@
         <v>194</v>
       </c>
       <c r="C80" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D80">
         <v>122</v>
@@ -39003,7 +38865,7 @@
         <v>194</v>
       </c>
       <c r="C81" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D81">
         <v>112</v>
@@ -39023,7 +38885,7 @@
         <v>194</v>
       </c>
       <c r="C82" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D82">
         <v>93</v>
@@ -39043,7 +38905,7 @@
         <v>194</v>
       </c>
       <c r="C83" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D83">
         <v>32</v>
@@ -39063,7 +38925,7 @@
         <v>194</v>
       </c>
       <c r="C84" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D84">
         <v>34</v>
@@ -39083,7 +38945,7 @@
         <v>194</v>
       </c>
       <c r="C85" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D85">
         <v>59</v>
@@ -39363,7 +39225,7 @@
         <v>112</v>
       </c>
       <c r="C99" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D99">
         <v>0</v>
@@ -39403,7 +39265,7 @@
         <v>112</v>
       </c>
       <c r="C101" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D101">
         <v>0</v>
@@ -39443,7 +39305,7 @@
         <v>112</v>
       </c>
       <c r="C103" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D103">
         <v>0</v>
@@ -39463,7 +39325,7 @@
         <v>112</v>
       </c>
       <c r="C104" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D104">
         <v>0</v>
@@ -39483,7 +39345,7 @@
         <v>112</v>
       </c>
       <c r="C105" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D105">
         <v>0</v>
@@ -39543,7 +39405,7 @@
         <v>112</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D108" s="3">
         <v>0</v>
@@ -39563,7 +39425,7 @@
         <v>112</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D109" s="3">
         <v>0</v>
@@ -39623,7 +39485,7 @@
         <v>112</v>
       </c>
       <c r="C112" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D112">
         <v>600</v>
@@ -39643,7 +39505,7 @@
         <v>112</v>
       </c>
       <c r="C113" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D113">
         <v>455</v>
@@ -39683,7 +39545,7 @@
         <v>112</v>
       </c>
       <c r="C115" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D115">
         <v>61</v>
@@ -39703,7 +39565,7 @@
         <v>112</v>
       </c>
       <c r="C116" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D116">
         <v>4</v>
@@ -39723,7 +39585,7 @@
         <v>112</v>
       </c>
       <c r="C117" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D117">
         <v>5</v>
@@ -39743,7 +39605,7 @@
         <v>112</v>
       </c>
       <c r="C118" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D118">
         <v>23</v>
@@ -39763,7 +39625,7 @@
         <v>112</v>
       </c>
       <c r="C119" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D119">
         <v>99</v>
@@ -39783,7 +39645,7 @@
         <v>112</v>
       </c>
       <c r="C120" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D120">
         <v>112</v>
@@ -39803,7 +39665,7 @@
         <v>112</v>
       </c>
       <c r="C121" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D121">
         <v>113</v>
@@ -39823,7 +39685,7 @@
         <v>112</v>
       </c>
       <c r="C122" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D122">
         <v>108</v>
@@ -39843,7 +39705,7 @@
         <v>112</v>
       </c>
       <c r="C123" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D123">
         <v>128</v>
@@ -39863,7 +39725,7 @@
         <v>112</v>
       </c>
       <c r="C124" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D124">
         <v>92</v>
@@ -39903,7 +39765,7 @@
         <v>112</v>
       </c>
       <c r="C126" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D126">
         <v>116</v>
@@ -39923,7 +39785,7 @@
         <v>112</v>
       </c>
       <c r="C127" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D127">
         <v>26</v>
@@ -39943,7 +39805,7 @@
         <v>112</v>
       </c>
       <c r="C128" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D128">
         <v>100</v>
@@ -39963,7 +39825,7 @@
         <v>112</v>
       </c>
       <c r="C129" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D129">
         <v>103</v>
@@ -39983,7 +39845,7 @@
         <v>112</v>
       </c>
       <c r="C130" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D130">
         <v>139</v>
@@ -40003,7 +39865,7 @@
         <v>112</v>
       </c>
       <c r="C131" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D131">
         <v>141</v>
@@ -40023,7 +39885,7 @@
         <v>112</v>
       </c>
       <c r="C132" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D132">
         <v>129</v>
@@ -40043,7 +39905,7 @@
         <v>112</v>
       </c>
       <c r="C133" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D133">
         <v>108</v>
@@ -40323,7 +40185,7 @@
         <v>196</v>
       </c>
       <c r="C147" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D147">
         <v>470</v>
@@ -40363,7 +40225,7 @@
         <v>196</v>
       </c>
       <c r="C149" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D149">
         <v>526</v>
@@ -40403,7 +40265,7 @@
         <v>196</v>
       </c>
       <c r="C151" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D151">
         <v>350</v>
@@ -40423,7 +40285,7 @@
         <v>196</v>
       </c>
       <c r="C152" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D152">
         <v>481</v>
@@ -40443,7 +40305,7 @@
         <v>196</v>
       </c>
       <c r="C153" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D153">
         <v>498</v>
@@ -40503,7 +40365,7 @@
         <v>196</v>
       </c>
       <c r="C156" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D156">
         <v>409</v>
@@ -40523,7 +40385,7 @@
         <v>196</v>
       </c>
       <c r="C157" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D157">
         <v>325</v>
@@ -40583,7 +40445,7 @@
         <v>196</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D160" s="3">
         <v>0</v>
@@ -40603,7 +40465,7 @@
         <v>196</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D161" s="3">
         <v>0</v>
@@ -40643,7 +40505,7 @@
         <v>196</v>
       </c>
       <c r="C163" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D163">
         <v>351</v>
@@ -40663,7 +40525,7 @@
         <v>196</v>
       </c>
       <c r="C164" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D164">
         <v>530</v>
@@ -40683,7 +40545,7 @@
         <v>196</v>
       </c>
       <c r="C165" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D165">
         <v>546</v>
@@ -40703,7 +40565,7 @@
         <v>196</v>
       </c>
       <c r="C166" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D166">
         <v>453</v>
@@ -40723,7 +40585,7 @@
         <v>196</v>
       </c>
       <c r="C167" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D167">
         <v>309</v>
@@ -40743,7 +40605,7 @@
         <v>196</v>
       </c>
       <c r="C168" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D168">
         <v>349</v>
@@ -40763,7 +40625,7 @@
         <v>196</v>
       </c>
       <c r="C169" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D169">
         <v>335</v>
@@ -40783,7 +40645,7 @@
         <v>196</v>
       </c>
       <c r="C170" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D170">
         <v>227</v>
@@ -40803,7 +40665,7 @@
         <v>196</v>
       </c>
       <c r="C171" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D171">
         <v>232</v>
@@ -40823,7 +40685,7 @@
         <v>196</v>
       </c>
       <c r="C172" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D172">
         <v>374</v>
@@ -40863,7 +40725,7 @@
         <v>196</v>
       </c>
       <c r="C174" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D174">
         <v>285</v>
@@ -40883,7 +40745,7 @@
         <v>196</v>
       </c>
       <c r="C175" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D175">
         <v>212</v>
@@ -40903,7 +40765,7 @@
         <v>196</v>
       </c>
       <c r="C176" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D176">
         <v>253</v>
@@ -40923,7 +40785,7 @@
         <v>196</v>
       </c>
       <c r="C177" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D177">
         <v>314</v>
@@ -40943,7 +40805,7 @@
         <v>196</v>
       </c>
       <c r="C178" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D178">
         <v>274</v>
@@ -40963,7 +40825,7 @@
         <v>196</v>
       </c>
       <c r="C179" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D179">
         <v>416</v>
@@ -40983,7 +40845,7 @@
         <v>196</v>
       </c>
       <c r="C180" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D180">
         <v>321</v>
@@ -41003,7 +40865,7 @@
         <v>196</v>
       </c>
       <c r="C181" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D181">
         <v>352</v>
@@ -41283,7 +41145,7 @@
         <v>127</v>
       </c>
       <c r="C195" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D195">
         <v>0</v>
@@ -41323,7 +41185,7 @@
         <v>127</v>
       </c>
       <c r="C197" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D197">
         <v>90.900000000001455</v>
@@ -41363,7 +41225,7 @@
         <v>127</v>
       </c>
       <c r="C199" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D199">
         <v>69.5</v>
@@ -41383,7 +41245,7 @@
         <v>127</v>
       </c>
       <c r="C200" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D200">
         <v>31.599999999999909</v>
@@ -41403,7 +41265,7 @@
         <v>127</v>
       </c>
       <c r="C201" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D201">
         <v>60.400000000000091</v>
@@ -41463,7 +41325,7 @@
         <v>127</v>
       </c>
       <c r="C204" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D204">
         <v>0</v>
@@ -41483,7 +41345,7 @@
         <v>127</v>
       </c>
       <c r="C205" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D205">
         <v>0</v>
@@ -41543,7 +41405,7 @@
         <v>127</v>
       </c>
       <c r="C208" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D208">
         <v>0</v>
@@ -41563,7 +41425,7 @@
         <v>127</v>
       </c>
       <c r="C209" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D209">
         <v>0</v>
@@ -41603,7 +41465,7 @@
         <v>127</v>
       </c>
       <c r="C211" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D211">
         <v>0</v>
@@ -41623,7 +41485,7 @@
         <v>127</v>
       </c>
       <c r="C212" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D212">
         <v>0</v>
@@ -41643,7 +41505,7 @@
         <v>127</v>
       </c>
       <c r="C213" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D213">
         <v>0</v>
@@ -41663,7 +41525,7 @@
         <v>127</v>
       </c>
       <c r="C214" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D214">
         <v>0</v>
@@ -41683,7 +41545,7 @@
         <v>127</v>
       </c>
       <c r="C215" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D215">
         <v>0</v>
@@ -41703,7 +41565,7 @@
         <v>127</v>
       </c>
       <c r="C216" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D216">
         <v>0</v>
@@ -41723,7 +41585,7 @@
         <v>127</v>
       </c>
       <c r="C217" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D217">
         <v>0</v>
@@ -41743,7 +41605,7 @@
         <v>127</v>
       </c>
       <c r="C218" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D218">
         <v>0</v>
@@ -41763,7 +41625,7 @@
         <v>127</v>
       </c>
       <c r="C219" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D219">
         <v>0</v>
@@ -41783,7 +41645,7 @@
         <v>127</v>
       </c>
       <c r="C220" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D220">
         <v>0</v>
@@ -41823,7 +41685,7 @@
         <v>127</v>
       </c>
       <c r="C222" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D222">
         <v>0</v>
@@ -41843,7 +41705,7 @@
         <v>127</v>
       </c>
       <c r="C223" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D223">
         <v>0</v>
@@ -41863,7 +41725,7 @@
         <v>127</v>
       </c>
       <c r="C224" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D224">
         <v>0</v>
@@ -41883,7 +41745,7 @@
         <v>127</v>
       </c>
       <c r="C225" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D225">
         <v>0</v>
@@ -41903,7 +41765,7 @@
         <v>127</v>
       </c>
       <c r="C226" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D226">
         <v>0</v>
@@ -41923,7 +41785,7 @@
         <v>127</v>
       </c>
       <c r="C227" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D227">
         <v>0</v>
@@ -41943,7 +41805,7 @@
         <v>127</v>
       </c>
       <c r="C228" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D228">
         <v>0</v>
@@ -41963,7 +41825,7 @@
         <v>127</v>
       </c>
       <c r="C229" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D229">
         <v>0</v>
@@ -42243,7 +42105,7 @@
         <v>118</v>
       </c>
       <c r="C243" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D243">
         <v>0</v>
@@ -42283,7 +42145,7 @@
         <v>118</v>
       </c>
       <c r="C245" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D245">
         <v>0</v>
@@ -42323,7 +42185,7 @@
         <v>118</v>
       </c>
       <c r="C247" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D247">
         <v>0</v>
@@ -42343,7 +42205,7 @@
         <v>118</v>
       </c>
       <c r="C248" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D248">
         <v>0</v>
@@ -42363,7 +42225,7 @@
         <v>118</v>
       </c>
       <c r="C249" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D249">
         <v>0</v>
@@ -42423,7 +42285,7 @@
         <v>118</v>
       </c>
       <c r="C252" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D252">
         <v>0</v>
@@ -42443,7 +42305,7 @@
         <v>118</v>
       </c>
       <c r="C253" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D253">
         <v>0</v>
@@ -42503,7 +42365,7 @@
         <v>118</v>
       </c>
       <c r="C256" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D256">
         <v>0</v>
@@ -42523,7 +42385,7 @@
         <v>118</v>
       </c>
       <c r="C257" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D257">
         <v>0</v>
@@ -42563,7 +42425,7 @@
         <v>118</v>
       </c>
       <c r="C259" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D259">
         <v>0</v>
@@ -42583,7 +42445,7 @@
         <v>118</v>
       </c>
       <c r="C260" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D260">
         <v>0</v>
@@ -42603,7 +42465,7 @@
         <v>118</v>
       </c>
       <c r="C261" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D261">
         <v>0</v>
@@ -42623,7 +42485,7 @@
         <v>118</v>
       </c>
       <c r="C262" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D262">
         <v>0</v>
@@ -42643,7 +42505,7 @@
         <v>118</v>
       </c>
       <c r="C263" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D263">
         <v>0</v>
@@ -42663,7 +42525,7 @@
         <v>118</v>
       </c>
       <c r="C264" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D264">
         <v>0</v>
@@ -42683,7 +42545,7 @@
         <v>118</v>
       </c>
       <c r="C265" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D265">
         <v>0</v>
@@ -42703,7 +42565,7 @@
         <v>118</v>
       </c>
       <c r="C266" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D266">
         <v>0</v>
@@ -42723,7 +42585,7 @@
         <v>118</v>
       </c>
       <c r="C267" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D267">
         <v>0</v>
@@ -42743,7 +42605,7 @@
         <v>118</v>
       </c>
       <c r="C268" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D268">
         <v>0</v>
@@ -42783,7 +42645,7 @@
         <v>118</v>
       </c>
       <c r="C270" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D270">
         <v>41.200000000000053</v>
@@ -42803,7 +42665,7 @@
         <v>118</v>
       </c>
       <c r="C271" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D271">
         <v>74.5</v>
@@ -42823,7 +42685,7 @@
         <v>118</v>
       </c>
       <c r="C272" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D272">
         <v>82.299999999999955</v>
@@ -42843,7 +42705,7 @@
         <v>118</v>
       </c>
       <c r="C273" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D273">
         <v>68.700000000000045</v>
@@ -42863,7 +42725,7 @@
         <v>118</v>
       </c>
       <c r="C274" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D274">
         <v>3.700000000000045</v>
@@ -42883,7 +42745,7 @@
         <v>118</v>
       </c>
       <c r="C275" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D275">
         <v>4.0999999999999091</v>
@@ -42903,7 +42765,7 @@
         <v>118</v>
       </c>
       <c r="C276" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D276">
         <v>0.90000000000009095</v>
@@ -42923,7 +42785,7 @@
         <v>118</v>
       </c>
       <c r="C277" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D277">
         <v>0</v>
@@ -43203,7 +43065,7 @@
         <v>119</v>
       </c>
       <c r="C291" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D291">
         <v>0</v>
@@ -43243,7 +43105,7 @@
         <v>119</v>
       </c>
       <c r="C293" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D293">
         <v>0</v>
@@ -43283,7 +43145,7 @@
         <v>119</v>
       </c>
       <c r="C295" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D295">
         <v>0</v>
@@ -43303,7 +43165,7 @@
         <v>119</v>
       </c>
       <c r="C296" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D296">
         <v>0</v>
@@ -43323,7 +43185,7 @@
         <v>119</v>
       </c>
       <c r="C297" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D297">
         <v>0</v>
@@ -43383,7 +43245,7 @@
         <v>119</v>
       </c>
       <c r="C300" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D300">
         <v>0</v>
@@ -43403,7 +43265,7 @@
         <v>119</v>
       </c>
       <c r="C301" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D301">
         <v>0</v>
@@ -43463,7 +43325,7 @@
         <v>119</v>
       </c>
       <c r="C304" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D304" s="3">
         <v>0</v>
@@ -43483,7 +43345,7 @@
         <v>119</v>
       </c>
       <c r="C305" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D305" s="3">
         <v>0</v>
@@ -43523,7 +43385,7 @@
         <v>119</v>
       </c>
       <c r="C307" s="3" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D307" s="3">
         <v>0</v>
@@ -43543,7 +43405,7 @@
         <v>119</v>
       </c>
       <c r="C308" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D308" s="3">
         <v>0</v>
@@ -43563,7 +43425,7 @@
         <v>119</v>
       </c>
       <c r="C309" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D309" s="3">
         <v>0</v>
@@ -43583,7 +43445,7 @@
         <v>119</v>
       </c>
       <c r="C310" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D310" s="3">
         <v>0</v>
@@ -43603,7 +43465,7 @@
         <v>119</v>
       </c>
       <c r="C311" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D311" s="3">
         <v>0</v>
@@ -43623,7 +43485,7 @@
         <v>119</v>
       </c>
       <c r="C312" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D312" s="3">
         <v>0</v>
@@ -43643,7 +43505,7 @@
         <v>119</v>
       </c>
       <c r="C313" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D313" s="3">
         <v>0</v>
@@ -43663,7 +43525,7 @@
         <v>119</v>
       </c>
       <c r="C314" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D314" s="3">
         <v>0</v>
@@ -43683,7 +43545,7 @@
         <v>119</v>
       </c>
       <c r="C315" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D315" s="3">
         <v>0</v>
@@ -43703,7 +43565,7 @@
         <v>119</v>
       </c>
       <c r="C316" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D316" s="3">
         <v>0</v>
@@ -43743,7 +43605,7 @@
         <v>119</v>
       </c>
       <c r="C318" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D318" s="3">
         <v>0</v>
@@ -43763,7 +43625,7 @@
         <v>119</v>
       </c>
       <c r="C319" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D319" s="3">
         <v>0</v>
@@ -43783,7 +43645,7 @@
         <v>119</v>
       </c>
       <c r="C320" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D320">
         <v>0</v>
@@ -43803,7 +43665,7 @@
         <v>119</v>
       </c>
       <c r="C321" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D321">
         <v>0</v>
@@ -43823,7 +43685,7 @@
         <v>119</v>
       </c>
       <c r="C322" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D322">
         <v>0</v>
@@ -43843,7 +43705,7 @@
         <v>119</v>
       </c>
       <c r="C323" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D323">
         <v>0</v>
@@ -43863,7 +43725,7 @@
         <v>119</v>
       </c>
       <c r="C324" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D324">
         <v>0</v>
@@ -43883,7 +43745,7 @@
         <v>119</v>
       </c>
       <c r="C325" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D325">
         <v>0</v>
@@ -44163,7 +44025,7 @@
         <v>120</v>
       </c>
       <c r="C339" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D339">
         <v>0</v>
@@ -44203,7 +44065,7 @@
         <v>120</v>
       </c>
       <c r="C341" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D341">
         <v>0</v>
@@ -44243,7 +44105,7 @@
         <v>120</v>
       </c>
       <c r="C343" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D343">
         <v>0</v>
@@ -44263,7 +44125,7 @@
         <v>120</v>
       </c>
       <c r="C344" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D344">
         <v>0</v>
@@ -44283,7 +44145,7 @@
         <v>120</v>
       </c>
       <c r="C345" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D345">
         <v>0</v>
@@ -44343,7 +44205,7 @@
         <v>120</v>
       </c>
       <c r="C348" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D348">
         <v>0</v>
@@ -44363,7 +44225,7 @@
         <v>120</v>
       </c>
       <c r="C349" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D349">
         <v>0</v>
@@ -44423,7 +44285,7 @@
         <v>120</v>
       </c>
       <c r="C352" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D352">
         <v>0</v>
@@ -44443,7 +44305,7 @@
         <v>120</v>
       </c>
       <c r="C353" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D353">
         <v>0</v>
@@ -44483,7 +44345,7 @@
         <v>120</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D355" s="2">
         <v>0</v>
@@ -44503,7 +44365,7 @@
         <v>120</v>
       </c>
       <c r="C356" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D356">
         <v>0</v>
@@ -44523,7 +44385,7 @@
         <v>120</v>
       </c>
       <c r="C357" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D357">
         <v>0</v>
@@ -44543,7 +44405,7 @@
         <v>120</v>
       </c>
       <c r="C358" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D358" s="3">
         <v>0</v>
@@ -44563,7 +44425,7 @@
         <v>120</v>
       </c>
       <c r="C359" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D359" s="3">
         <v>0</v>
@@ -44583,7 +44445,7 @@
         <v>120</v>
       </c>
       <c r="C360" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D360" s="3">
         <v>0</v>
@@ -44603,7 +44465,7 @@
         <v>120</v>
       </c>
       <c r="C361" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D361">
         <v>0</v>
@@ -44623,7 +44485,7 @@
         <v>120</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D362" s="2">
         <v>0</v>
@@ -44643,7 +44505,7 @@
         <v>120</v>
       </c>
       <c r="C363" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D363">
         <v>0</v>
@@ -44663,7 +44525,7 @@
         <v>120</v>
       </c>
       <c r="C364" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D364">
         <v>0</v>
@@ -44703,7 +44565,7 @@
         <v>120</v>
       </c>
       <c r="C366" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D366">
         <v>0</v>
@@ -44723,7 +44585,7 @@
         <v>120</v>
       </c>
       <c r="C367" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D367">
         <v>0</v>
@@ -44743,7 +44605,7 @@
         <v>120</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D368" s="2">
         <v>0</v>
@@ -44763,7 +44625,7 @@
         <v>120</v>
       </c>
       <c r="C369" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D369">
         <v>0</v>
@@ -44783,7 +44645,7 @@
         <v>120</v>
       </c>
       <c r="C370" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D370">
         <v>0</v>
@@ -44803,7 +44665,7 @@
         <v>120</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D371" s="2">
         <v>0</v>
@@ -44823,7 +44685,7 @@
         <v>120</v>
       </c>
       <c r="C372" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D372">
         <v>0</v>
@@ -44843,7 +44705,7 @@
         <v>120</v>
       </c>
       <c r="C373" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D373">
         <v>0</v>
@@ -45123,7 +44985,7 @@
         <v>121</v>
       </c>
       <c r="C387" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D387" s="3">
         <v>0</v>
@@ -45163,7 +45025,7 @@
         <v>121</v>
       </c>
       <c r="C389" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D389" s="3">
         <v>0</v>
@@ -45203,7 +45065,7 @@
         <v>121</v>
       </c>
       <c r="C391" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D391" s="3">
         <v>0</v>
@@ -45223,7 +45085,7 @@
         <v>121</v>
       </c>
       <c r="C392" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D392" s="3">
         <v>0</v>
@@ -45243,7 +45105,7 @@
         <v>121</v>
       </c>
       <c r="C393" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D393" s="3">
         <v>0</v>
@@ -45303,7 +45165,7 @@
         <v>121</v>
       </c>
       <c r="C396" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D396" s="3">
         <v>0</v>
@@ -45323,7 +45185,7 @@
         <v>121</v>
       </c>
       <c r="C397" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D397" s="3">
         <v>0</v>
@@ -45383,7 +45245,7 @@
         <v>121</v>
       </c>
       <c r="C400" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D400">
         <v>18</v>
@@ -45403,7 +45265,7 @@
         <v>121</v>
       </c>
       <c r="C401" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D401" s="3">
         <v>0</v>
@@ -45443,7 +45305,7 @@
         <v>121</v>
       </c>
       <c r="C403" s="3" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D403" s="3">
         <v>0</v>
@@ -45463,7 +45325,7 @@
         <v>121</v>
       </c>
       <c r="C404" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D404" s="3">
         <v>0</v>
@@ -45483,7 +45345,7 @@
         <v>121</v>
       </c>
       <c r="C405" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D405" s="3">
         <v>0</v>
@@ -45503,7 +45365,7 @@
         <v>121</v>
       </c>
       <c r="C406" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D406" s="3">
         <v>0</v>
@@ -45523,7 +45385,7 @@
         <v>121</v>
       </c>
       <c r="C407" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D407" s="3">
         <v>0</v>
@@ -45543,7 +45405,7 @@
         <v>121</v>
       </c>
       <c r="C408" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D408" s="3">
         <v>0</v>
@@ -45563,7 +45425,7 @@
         <v>121</v>
       </c>
       <c r="C409" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D409" s="3">
         <v>0</v>
@@ -45583,7 +45445,7 @@
         <v>121</v>
       </c>
       <c r="C410" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D410" s="3">
         <v>0</v>
@@ -45603,7 +45465,7 @@
         <v>121</v>
       </c>
       <c r="C411" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D411" s="3">
         <v>0</v>
@@ -45623,7 +45485,7 @@
         <v>121</v>
       </c>
       <c r="C412" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D412" s="3">
         <v>0</v>
@@ -45663,7 +45525,7 @@
         <v>121</v>
       </c>
       <c r="C414" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D414">
         <v>0</v>
@@ -45683,7 +45545,7 @@
         <v>121</v>
       </c>
       <c r="C415" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D415">
         <v>0</v>
@@ -45703,7 +45565,7 @@
         <v>121</v>
       </c>
       <c r="C416" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D416">
         <v>0</v>
@@ -45723,7 +45585,7 @@
         <v>121</v>
       </c>
       <c r="C417" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D417">
         <v>0</v>
@@ -45743,7 +45605,7 @@
         <v>121</v>
       </c>
       <c r="C418" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D418">
         <v>0</v>
@@ -45763,7 +45625,7 @@
         <v>121</v>
       </c>
       <c r="C419" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D419">
         <v>0</v>
@@ -45783,7 +45645,7 @@
         <v>121</v>
       </c>
       <c r="C420" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D420">
         <v>0</v>
@@ -45803,7 +45665,7 @@
         <v>121</v>
       </c>
       <c r="C421" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D421">
         <v>0</v>
@@ -46083,7 +45945,7 @@
         <v>172</v>
       </c>
       <c r="C435" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D435">
         <v>7</v>
@@ -46123,7 +45985,7 @@
         <v>172</v>
       </c>
       <c r="C437" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D437">
         <v>14</v>
@@ -46163,7 +46025,7 @@
         <v>172</v>
       </c>
       <c r="C439" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D439">
         <v>48</v>
@@ -46183,7 +46045,7 @@
         <v>172</v>
       </c>
       <c r="C440" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D440">
         <v>15</v>
@@ -46203,7 +46065,7 @@
         <v>172</v>
       </c>
       <c r="C441" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D441">
         <v>31</v>
@@ -46263,7 +46125,7 @@
         <v>172</v>
       </c>
       <c r="C444" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D444">
         <v>0</v>
@@ -46283,7 +46145,7 @@
         <v>172</v>
       </c>
       <c r="C445" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D445">
         <v>11</v>
@@ -46343,7 +46205,7 @@
         <v>172</v>
       </c>
       <c r="C448" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D448">
         <v>0</v>
@@ -46363,7 +46225,7 @@
         <v>172</v>
       </c>
       <c r="C449" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D449">
         <v>0</v>
@@ -46403,7 +46265,7 @@
         <v>172</v>
       </c>
       <c r="C451" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D451">
         <v>4</v>
@@ -46423,7 +46285,7 @@
         <v>172</v>
       </c>
       <c r="C452" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D452">
         <v>44</v>
@@ -46443,7 +46305,7 @@
         <v>172</v>
       </c>
       <c r="C453" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D453">
         <v>28</v>
@@ -46463,7 +46325,7 @@
         <v>172</v>
       </c>
       <c r="C454" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D454">
         <v>26</v>
@@ -46483,7 +46345,7 @@
         <v>172</v>
       </c>
       <c r="C455" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D455">
         <v>30</v>
@@ -46503,7 +46365,7 @@
         <v>172</v>
       </c>
       <c r="C456" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D456">
         <v>22</v>
@@ -46523,7 +46385,7 @@
         <v>172</v>
       </c>
       <c r="C457" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D457">
         <v>38</v>
@@ -46543,7 +46405,7 @@
         <v>172</v>
       </c>
       <c r="C458" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D458">
         <v>22</v>
@@ -46563,7 +46425,7 @@
         <v>172</v>
       </c>
       <c r="C459" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D459">
         <v>4</v>
@@ -46583,7 +46445,7 @@
         <v>172</v>
       </c>
       <c r="C460" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D460">
         <v>41</v>
@@ -46623,7 +46485,7 @@
         <v>172</v>
       </c>
       <c r="C462" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D462">
         <v>30</v>
@@ -46643,7 +46505,7 @@
         <v>172</v>
       </c>
       <c r="C463" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D463">
         <v>13</v>
@@ -46663,7 +46525,7 @@
         <v>172</v>
       </c>
       <c r="C464" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D464">
         <v>43</v>
@@ -46683,7 +46545,7 @@
         <v>172</v>
       </c>
       <c r="C465" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D465">
         <v>0</v>
@@ -46703,7 +46565,7 @@
         <v>172</v>
       </c>
       <c r="C466" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D466">
         <v>0</v>
@@ -46723,7 +46585,7 @@
         <v>172</v>
       </c>
       <c r="C467" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D467">
         <v>0</v>
@@ -46743,7 +46605,7 @@
         <v>172</v>
       </c>
       <c r="C468" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D468" s="2">
         <v>0</v>
@@ -46763,7 +46625,7 @@
         <v>172</v>
       </c>
       <c r="C469" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D469">
         <v>0</v>
@@ -47043,7 +46905,7 @@
         <v>49</v>
       </c>
       <c r="C483" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D483">
         <v>8</v>
@@ -47083,7 +46945,7 @@
         <v>49</v>
       </c>
       <c r="C485" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D485">
         <v>7</v>
@@ -47123,7 +46985,7 @@
         <v>49</v>
       </c>
       <c r="C487" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D487">
         <v>20</v>
@@ -47143,7 +47005,7 @@
         <v>49</v>
       </c>
       <c r="C488" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D488">
         <v>34</v>
@@ -47163,7 +47025,7 @@
         <v>49</v>
       </c>
       <c r="C489" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D489">
         <v>8</v>
@@ -47223,7 +47085,7 @@
         <v>49</v>
       </c>
       <c r="C492" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D492">
         <v>12</v>
@@ -47243,7 +47105,7 @@
         <v>49</v>
       </c>
       <c r="C493" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D493">
         <v>3</v>
@@ -47303,7 +47165,7 @@
         <v>49</v>
       </c>
       <c r="C496" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D496">
         <v>35</v>
@@ -47323,7 +47185,7 @@
         <v>49</v>
       </c>
       <c r="C497" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D497">
         <v>31</v>
@@ -47363,7 +47225,7 @@
         <v>49</v>
       </c>
       <c r="C499" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D499">
         <v>7</v>
@@ -47383,7 +47245,7 @@
         <v>49</v>
       </c>
       <c r="C500" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D500">
         <v>3</v>
@@ -47403,7 +47265,7 @@
         <v>49</v>
       </c>
       <c r="C501" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D501">
         <v>0</v>
@@ -47423,7 +47285,7 @@
         <v>49</v>
       </c>
       <c r="C502" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D502">
         <v>0</v>
@@ -47443,7 +47305,7 @@
         <v>49</v>
       </c>
       <c r="C503" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D503">
         <v>0</v>
@@ -47463,7 +47325,7 @@
         <v>49</v>
       </c>
       <c r="C504" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D504" s="2">
         <v>0</v>
@@ -47483,7 +47345,7 @@
         <v>49</v>
       </c>
       <c r="C505" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D505">
         <v>0</v>
@@ -47503,7 +47365,7 @@
         <v>49</v>
       </c>
       <c r="C506" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D506">
         <v>0</v>
@@ -47523,7 +47385,7 @@
         <v>49</v>
       </c>
       <c r="C507" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D507">
         <v>0</v>
@@ -47543,7 +47405,7 @@
         <v>49</v>
       </c>
       <c r="C508" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D508">
         <v>0</v>
@@ -47583,7 +47445,7 @@
         <v>49</v>
       </c>
       <c r="C510" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D510">
         <v>26.600000000000019</v>
@@ -47603,7 +47465,7 @@
         <v>49</v>
       </c>
       <c r="C511" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D511">
         <v>33.299999999999947</v>
@@ -47623,7 +47485,7 @@
         <v>49</v>
       </c>
       <c r="C512" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D512">
         <v>31.200000000000049</v>
@@ -47643,7 +47505,7 @@
         <v>49</v>
       </c>
       <c r="C513" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D513">
         <v>46.899999999999977</v>
@@ -47663,7 +47525,7 @@
         <v>49</v>
       </c>
       <c r="C514" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D514">
         <v>25</v>
@@ -47683,7 +47545,7 @@
         <v>49</v>
       </c>
       <c r="C515" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D515">
         <v>48.5</v>
@@ -47703,7 +47565,7 @@
         <v>49</v>
       </c>
       <c r="C516" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D516">
         <v>38.799999999999947</v>
@@ -47723,7 +47585,7 @@
         <v>49</v>
       </c>
       <c r="C517" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D517">
         <v>32</v>
@@ -48003,7 +47865,7 @@
         <v>122</v>
       </c>
       <c r="C531" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D531">
         <v>0</v>
@@ -48043,7 +47905,7 @@
         <v>122</v>
       </c>
       <c r="C533" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D533">
         <v>0</v>
@@ -48083,7 +47945,7 @@
         <v>122</v>
       </c>
       <c r="C535" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D535">
         <v>0</v>
@@ -48103,7 +47965,7 @@
         <v>122</v>
       </c>
       <c r="C536" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D536">
         <v>0</v>
@@ -48123,7 +47985,7 @@
         <v>122</v>
       </c>
       <c r="C537" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D537">
         <v>0</v>
@@ -48183,7 +48045,7 @@
         <v>122</v>
       </c>
       <c r="C540" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D540">
         <v>0</v>
@@ -48203,7 +48065,7 @@
         <v>122</v>
       </c>
       <c r="C541" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D541">
         <v>0</v>
@@ -48263,7 +48125,7 @@
         <v>122</v>
       </c>
       <c r="C544" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D544">
         <v>0</v>
@@ -48283,7 +48145,7 @@
         <v>122</v>
       </c>
       <c r="C545" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D545">
         <v>0</v>
@@ -48323,7 +48185,7 @@
         <v>122</v>
       </c>
       <c r="C547" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D547">
         <v>0</v>
@@ -48343,7 +48205,7 @@
         <v>122</v>
       </c>
       <c r="C548" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D548">
         <v>0</v>
@@ -48363,7 +48225,7 @@
         <v>122</v>
       </c>
       <c r="C549" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D549">
         <v>0</v>
@@ -48383,7 +48245,7 @@
         <v>122</v>
       </c>
       <c r="C550" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D550">
         <v>0</v>
@@ -48403,7 +48265,7 @@
         <v>122</v>
       </c>
       <c r="C551" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D551">
         <v>0</v>
@@ -48423,7 +48285,7 @@
         <v>122</v>
       </c>
       <c r="C552" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D552">
         <v>0</v>
@@ -48443,7 +48305,7 @@
         <v>122</v>
       </c>
       <c r="C553" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D553">
         <v>0</v>
@@ -48463,7 +48325,7 @@
         <v>122</v>
       </c>
       <c r="C554" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D554">
         <v>0</v>
@@ -48483,7 +48345,7 @@
         <v>122</v>
       </c>
       <c r="C555" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D555">
         <v>0</v>
@@ -48503,7 +48365,7 @@
         <v>122</v>
       </c>
       <c r="C556" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D556" s="2">
         <v>0</v>
@@ -48543,7 +48405,7 @@
         <v>122</v>
       </c>
       <c r="C558" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D558">
         <v>0</v>
@@ -48563,7 +48425,7 @@
         <v>122</v>
       </c>
       <c r="C559" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D559">
         <v>0</v>
@@ -48583,7 +48445,7 @@
         <v>122</v>
       </c>
       <c r="C560" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D560">
         <v>25</v>
@@ -48603,7 +48465,7 @@
         <v>122</v>
       </c>
       <c r="C561" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D561">
         <v>20</v>
@@ -48623,7 +48485,7 @@
         <v>122</v>
       </c>
       <c r="C562" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D562">
         <v>38</v>
@@ -48643,7 +48505,7 @@
         <v>122</v>
       </c>
       <c r="C563" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D563">
         <v>69</v>
@@ -48663,7 +48525,7 @@
         <v>122</v>
       </c>
       <c r="C564" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D564">
         <v>94</v>
@@ -48683,7 +48545,7 @@
         <v>122</v>
       </c>
       <c r="C565" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D565">
         <v>79</v>

</xml_diff>